<commit_message>
[updated] Agregar link de los prototipos a la matriz
</commit_message>
<xml_diff>
--- a/documentacion/matriz-trazabilidad.xlsx
+++ b/documentacion/matriz-trazabilidad.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="132">
   <si>
     <t>ID</t>
   </si>
@@ -32,7 +32,7 @@
     <t>Historias de Usuario</t>
   </si>
   <si>
-    <t>Dependencias</t>
+    <t>Prototipo</t>
   </si>
   <si>
     <t>Pruebas</t>
@@ -59,7 +59,13 @@
     <t>CF-7</t>
   </si>
   <si>
-    <t>Frontend (Bootstrap)</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-inicio.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>POR HACER</t>
@@ -77,7 +83,13 @@
     <t>CF-8</t>
   </si>
   <si>
-    <t>Frontend</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-inicio.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-3</t>
@@ -92,7 +104,13 @@
     <t>CF-9</t>
   </si>
   <si>
-    <t>Bootstrap responsive</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-4</t>
@@ -104,6 +122,15 @@
     <t>CF-11</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
+  </si>
+  <si>
     <t>RF-5</t>
   </si>
   <si>
@@ -113,6 +140,15 @@
     <t>Todos</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
+  </si>
+  <si>
     <t>RF-6</t>
   </si>
   <si>
@@ -125,7 +161,13 @@
     <t>CF-12</t>
   </si>
   <si>
-    <t>Backend + MongoDB</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-7</t>
@@ -134,7 +176,13 @@
     <t>Campos obligatorios del formulario de inscripción</t>
   </si>
   <si>
-    <t>Validación backend</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-8</t>
@@ -146,7 +194,13 @@
     <t>CF-10</t>
   </si>
   <si>
-    <t>Backend queries</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-9</t>
@@ -155,7 +209,13 @@
     <t>Búsqueda de actividades por nombre</t>
   </si>
   <si>
-    <t>Backend search</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-10</t>
@@ -167,7 +227,13 @@
     <t>CF-13</t>
   </si>
   <si>
-    <t>Frontend routing</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-11</t>
@@ -182,7 +248,13 @@
     <t>CF-14</t>
   </si>
   <si>
-    <t>Backend sorting</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-12</t>
@@ -191,7 +263,13 @@
     <t>Página detalle de actividad completa</t>
   </si>
   <si>
-    <t>Backend + DB</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-detalles-actividad.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-13</t>
@@ -200,7 +278,13 @@
     <t>Filtros de agenda por fecha y eventos futuros (+8h)</t>
   </si>
   <si>
-    <t>Backend lógica de tiempo</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-14</t>
@@ -209,7 +293,13 @@
     <t>Botón de detalle en agenda</t>
   </si>
   <si>
-    <t>Routing frontend</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-15</t>
@@ -224,7 +314,13 @@
     <t>CF-15</t>
   </si>
   <si>
-    <t>Backend</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-16</t>
@@ -233,7 +329,13 @@
     <t>Información de cada stand</t>
   </si>
   <si>
-    <t>DB MongoDB</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-17</t>
@@ -242,7 +344,13 @@
     <t>Control de inscripción según disponibilidad y tiempo</t>
   </si>
   <si>
-    <t>Backend reglas negocio</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-18</t>
@@ -257,7 +365,13 @@
     <t>CF-22</t>
   </si>
   <si>
-    <t>Auth + backend</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-19</t>
@@ -266,7 +380,13 @@
     <t>Opciones admin en tarjetas (editar/eliminar)</t>
   </si>
   <si>
-    <t>Auth</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-20</t>
@@ -278,7 +398,13 @@
     <t>CF-24</t>
   </si>
   <si>
-    <t>Backend validation</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-21</t>
@@ -293,7 +419,13 @@
     <t>CF-25</t>
   </si>
   <si>
-    <t>Frontend JS</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-22</t>
@@ -302,6 +434,15 @@
     <t>Footer con contacto + formulario emergente</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
+  </si>
+  <si>
     <t>RF-23</t>
   </si>
   <si>
@@ -311,7 +452,13 @@
     <t>CF-26</t>
   </si>
   <si>
-    <t>Backend email service</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-24</t>
@@ -323,7 +470,13 @@
     <t>CF-33</t>
   </si>
   <si>
-    <t>Backend + Auth</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RF-25</t>
@@ -332,7 +485,13 @@
     <t>Creación de stands por admin</t>
   </si>
   <si>
-    <t>Casos de prueba</t>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
+    </r>
   </si>
   <si>
     <t>RNF-1</t>
@@ -405,7 +564,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -422,6 +581,10 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -462,8 +625,8 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
@@ -690,11 +853,11 @@
     <col customWidth="1" min="1" max="1" width="5.63"/>
     <col customWidth="1" min="3" max="3" width="52.38"/>
     <col customWidth="1" min="5" max="5" width="17.75"/>
-    <col customWidth="1" min="6" max="7" width="20.13"/>
-    <col customWidth="1" min="8" max="8" width="28.38"/>
+    <col customWidth="1" min="6" max="8" width="20.13"/>
+    <col customWidth="1" min="9" max="9" width="10.88"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -742,7 +905,7 @@
       <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H2" s="2"/>
@@ -769,7 +932,7 @@
       <c r="F3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>21</v>
       </c>
       <c r="H3" s="2"/>
@@ -796,7 +959,7 @@
       <c r="F4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>26</v>
       </c>
       <c r="H4" s="2"/>
@@ -823,8 +986,8 @@
       <c r="F5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>21</v>
+      <c r="G5" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -833,16 +996,16 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>13</v>
@@ -850,8 +1013,8 @@
       <c r="F6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>21</v>
+      <c r="G6" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -860,25 +1023,25 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -887,25 +1050,25 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -914,13 +1077,13 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>12</v>
@@ -929,10 +1092,10 @@
         <v>24</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -941,13 +1104,13 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>12</v>
@@ -956,10 +1119,10 @@
         <v>24</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -968,13 +1131,13 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>12</v>
@@ -983,10 +1146,10 @@
         <v>24</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -995,25 +1158,25 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -1022,13 +1185,13 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>12</v>
@@ -1039,8 +1202,8 @@
       <c r="F13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>59</v>
+      <c r="G13" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -1049,25 +1212,25 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -1076,25 +1239,25 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>65</v>
+        <v>56</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -1103,25 +1266,25 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
@@ -1130,25 +1293,25 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
@@ -1157,25 +1320,25 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>76</v>
+        <v>38</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
@@ -1184,25 +1347,25 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
@@ -1211,25 +1374,25 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2" t="s">
@@ -1238,25 +1401,25 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>90</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
@@ -1265,25 +1428,25 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2" t="s">
@@ -1292,25 +1455,25 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>21</v>
+        <v>94</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2" t="s">
@@ -1319,25 +1482,25 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2" t="s">
@@ -1346,25 +1509,25 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2" t="s">
@@ -1373,25 +1536,25 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>70</v>
+      <c r="G26" s="3" t="s">
+        <v>109</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2" t="s">
@@ -1399,7 +1562,34 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="G2"/>
+    <hyperlink r:id="rId2" ref="G3"/>
+    <hyperlink r:id="rId3" ref="G4"/>
+    <hyperlink r:id="rId4" ref="G5"/>
+    <hyperlink r:id="rId5" ref="G6"/>
+    <hyperlink r:id="rId6" ref="G7"/>
+    <hyperlink r:id="rId7" ref="G8"/>
+    <hyperlink r:id="rId8" ref="G9"/>
+    <hyperlink r:id="rId9" ref="G10"/>
+    <hyperlink r:id="rId10" ref="G11"/>
+    <hyperlink r:id="rId11" ref="G12"/>
+    <hyperlink r:id="rId12" ref="G13"/>
+    <hyperlink r:id="rId13" ref="G14"/>
+    <hyperlink r:id="rId14" ref="G15"/>
+    <hyperlink r:id="rId15" ref="G16"/>
+    <hyperlink r:id="rId16" ref="G17"/>
+    <hyperlink r:id="rId17" ref="G18"/>
+    <hyperlink r:id="rId18" ref="G19"/>
+    <hyperlink r:id="rId19" ref="G20"/>
+    <hyperlink r:id="rId20" ref="G21"/>
+    <hyperlink r:id="rId21" ref="G22"/>
+    <hyperlink r:id="rId22" ref="G23"/>
+    <hyperlink r:id="rId23" ref="G24"/>
+    <hyperlink r:id="rId24" ref="G25"/>
+    <hyperlink r:id="rId25" ref="G26"/>
+  </hyperlinks>
+  <drawing r:id="rId26"/>
 </worksheet>
 </file>
 
@@ -1433,7 +1623,7 @@
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>106</v>
+        <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
@@ -1441,16 +1631,16 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>20</v>
@@ -1462,19 +1652,19 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="2" t="s">
@@ -1483,19 +1673,19 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="2" t="s">
@@ -1504,19 +1694,19 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="2" t="s">
@@ -1525,19 +1715,19 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="2" t="s">
@@ -1546,19 +1736,19 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="2" t="s">
@@ -1567,19 +1757,19 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="2" t="s">
@@ -1588,19 +1778,19 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="2" t="s">

</xml_diff>

<commit_message>
[updated] Actualizacion del eds y matriz de trazabilidad. [new] agregar diagramas de arquitectura y diseno de entidades
</commit_message>
<xml_diff>
--- a/documentacion/matriz-trazabilidad.xlsx
+++ b/documentacion/matriz-trazabilidad.xlsx
@@ -1,18 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/af297d4d3962f505/Documents/CENFOTEC/Proyecto Integrador 1/SOFT-11-CampusFest/documentacion/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_CA882769DC6245E6C57594C85769F60CCA80B693" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C6847C3-E2C2-4D15-B3E6-8B3F363077D9}"/>
+  <bookViews>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Funcionales" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="No Funcionales" sheetId="2" r:id="rId6"/>
+    <sheet name="Funcionales" sheetId="1" r:id="rId1"/>
+    <sheet name="No Funcionales" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="136">
   <si>
     <t>ID</t>
   </si>
@@ -61,8 +70,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-inicio.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -85,8 +96,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-inicio.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -106,8 +119,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -124,8 +139,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -142,8 +159,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -163,8 +182,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -178,8 +199,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -196,8 +219,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -211,8 +236,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -229,8 +256,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -250,8 +279,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -265,8 +296,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-detalles-actividad.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -280,8 +313,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -295,8 +330,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-agenda.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -316,8 +353,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -331,8 +370,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -346,8 +387,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-inscripcion.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -367,8 +410,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -382,8 +427,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -400,8 +447,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-actividades.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -421,8 +470,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -436,8 +487,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -454,8 +507,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-formulario-contacto.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -472,8 +527,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -487,8 +544,10 @@
   <si>
     <r>
       <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
       </rPr>
       <t>SOFT-11-CampusFest/documentacion/UI/prototipo-stands.pdf at main · verbrannt-bob/SOFT-11-CampusFest</t>
     </r>
@@ -558,33 +617,55 @@
   </si>
   <si>
     <t>Uso de paleta oficial U Cenfotec</t>
+  </si>
+  <si>
+    <t>EndPoint</t>
+  </si>
+  <si>
+    <t>/actividades</t>
+  </si>
+  <si>
+    <t>/visitantes</t>
+  </si>
+  <si>
+    <t>/stands</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -592,11 +673,17 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -610,39 +697,34 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,7 +732,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -840,24 +922,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="5.63"/>
-    <col customWidth="1" min="3" max="3" width="52.38"/>
-    <col customWidth="1" min="5" max="5" width="17.75"/>
-    <col customWidth="1" min="6" max="8" width="20.13"/>
-    <col customWidth="1" min="9" max="9" width="10.88"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
+    <col min="3" max="3" width="52.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="8" width="20.140625" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.0" customHeight="1">
+    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -885,8 +970,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="J1" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -912,8 +1000,9 @@
       <c r="I2" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -939,8 +1028,9 @@
       <c r="I3" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -966,8 +1056,9 @@
       <c r="I4" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -993,8 +1084,11 @@
       <c r="I5" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="J5" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -1020,8 +1114,9 @@
       <c r="I6" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -1047,8 +1142,11 @@
       <c r="I7" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="J7" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -1074,8 +1172,11 @@
       <c r="I8" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="J8" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>43</v>
       </c>
@@ -1101,8 +1202,11 @@
       <c r="I9" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="J9" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>47</v>
       </c>
@@ -1128,8 +1232,11 @@
       <c r="I10" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="J10" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -1155,8 +1262,11 @@
       <c r="I11" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="J11" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>54</v>
       </c>
@@ -1182,8 +1292,11 @@
       <c r="I12" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="13">
+      <c r="J12" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>59</v>
       </c>
@@ -1209,8 +1322,11 @@
       <c r="I13" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="J13" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>62</v>
       </c>
@@ -1236,8 +1352,11 @@
       <c r="I14" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15">
+      <c r="J14" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>65</v>
       </c>
@@ -1263,8 +1382,11 @@
       <c r="I15" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16">
+      <c r="J15" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>68</v>
       </c>
@@ -1290,8 +1412,11 @@
       <c r="I16" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17">
+      <c r="J16" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>73</v>
       </c>
@@ -1317,8 +1442,11 @@
       <c r="I17" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18">
+      <c r="J17" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>76</v>
       </c>
@@ -1344,8 +1472,11 @@
       <c r="I18" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19">
+      <c r="J18" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>79</v>
       </c>
@@ -1371,8 +1502,11 @@
       <c r="I19" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20">
+      <c r="J19" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>84</v>
       </c>
@@ -1398,8 +1532,11 @@
       <c r="I20" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="21">
+      <c r="J20" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>87</v>
       </c>
@@ -1425,8 +1562,11 @@
       <c r="I21" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="22">
+      <c r="J21" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>91</v>
       </c>
@@ -1452,8 +1592,9 @@
       <c r="I22" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>96</v>
       </c>
@@ -1479,8 +1620,9 @@
       <c r="I23" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24">
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>99</v>
       </c>
@@ -1506,8 +1648,9 @@
       <c r="I24" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="25">
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>103</v>
       </c>
@@ -1533,8 +1676,11 @@
       <c r="I25" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26">
+      <c r="J25" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>107</v>
       </c>
@@ -1560,53 +1706,57 @@
       <c r="I26" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="J26" s="2" t="s">
+        <v>135</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="G2"/>
-    <hyperlink r:id="rId2" ref="G3"/>
-    <hyperlink r:id="rId3" ref="G4"/>
-    <hyperlink r:id="rId4" ref="G5"/>
-    <hyperlink r:id="rId5" ref="G6"/>
-    <hyperlink r:id="rId6" ref="G7"/>
-    <hyperlink r:id="rId7" ref="G8"/>
-    <hyperlink r:id="rId8" ref="G9"/>
-    <hyperlink r:id="rId9" ref="G10"/>
-    <hyperlink r:id="rId10" ref="G11"/>
-    <hyperlink r:id="rId11" ref="G12"/>
-    <hyperlink r:id="rId12" ref="G13"/>
-    <hyperlink r:id="rId13" ref="G14"/>
-    <hyperlink r:id="rId14" ref="G15"/>
-    <hyperlink r:id="rId15" ref="G16"/>
-    <hyperlink r:id="rId16" ref="G17"/>
-    <hyperlink r:id="rId17" ref="G18"/>
-    <hyperlink r:id="rId18" ref="G19"/>
-    <hyperlink r:id="rId19" ref="G20"/>
-    <hyperlink r:id="rId20" ref="G21"/>
-    <hyperlink r:id="rId21" ref="G22"/>
-    <hyperlink r:id="rId22" ref="G23"/>
-    <hyperlink r:id="rId23" ref="G24"/>
-    <hyperlink r:id="rId24" ref="G25"/>
-    <hyperlink r:id="rId25" ref="G26"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="G11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="G12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="G13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="G15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="G16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="G17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="G18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="G19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="G20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="G21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="G22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="G23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="G24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="G25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="G26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
   </hyperlinks>
-  <drawing r:id="rId26"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="33.5"/>
-    <col customWidth="1" min="4" max="4" width="12.88"/>
-    <col customWidth="1" min="5" max="5" width="17.25"/>
-    <col customWidth="1" min="6" max="6" width="14.38"/>
+    <col min="3" max="3" width="33.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1629,7 +1779,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>110</v>
       </c>
@@ -1645,12 +1795,12 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="4"/>
+      <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>114</v>
       </c>
@@ -1666,12 +1816,12 @@
       <c r="E3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>117</v>
       </c>
@@ -1687,12 +1837,12 @@
       <c r="E4" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>121</v>
       </c>
@@ -1708,12 +1858,12 @@
       <c r="E5" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>123</v>
       </c>
@@ -1729,12 +1879,12 @@
       <c r="E6" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>125</v>
       </c>
@@ -1750,12 +1900,12 @@
       <c r="E7" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>127</v>
       </c>
@@ -1771,12 +1921,12 @@
       <c r="E8" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>130</v>
       </c>
@@ -1792,12 +1942,12 @@
       <c r="E9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>